<commit_message>
Added notes file for tracking
</commit_message>
<xml_diff>
--- a/sync/prayer_db.xlsx
+++ b/sync/prayer_db.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>14:42</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:42</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>14:46</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1995,7 +1995,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:04</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:14</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>15:16</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>15:17</t>
+          <t>15:16</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:17</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>15:29</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -4139,7 +4139,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:29</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>15:31</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>15:32</t>
+          <t>15:31</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:37</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>16:42</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>16:54</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6417,7 +6417,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:54</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>17:02</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7623,7 +7623,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>17:06</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8628,7 +8628,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>17:09</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -9164,7 +9164,7 @@
       </c>
       <c r="H131" t="inlineStr">
         <is>
-          <t>17:13</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:13</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -10102,7 +10102,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>17:18</t>
+          <t>17:17</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -10303,7 +10303,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>17:19</t>
+          <t>17:18</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -10906,7 +10906,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
@@ -12581,7 +12581,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>17:27</t>
+          <t>17:28</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
@@ -13653,7 +13653,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>17:27</t>
+          <t>17:28</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
@@ -14792,7 +14792,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -14926,7 +14926,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -15663,7 +15663,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="I228" t="inlineStr">
@@ -15931,7 +15931,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -17271,7 +17271,7 @@
       </c>
       <c r="H252" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="I252" t="inlineStr">
@@ -17338,7 +17338,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -17673,7 +17673,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -17941,7 +17941,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>16:39</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -18209,7 +18209,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -18410,7 +18410,7 @@
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:31</t>
         </is>
       </c>
       <c r="I269" t="inlineStr">
@@ -18678,7 +18678,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:26</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -18879,7 +18879,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:22</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -19080,7 +19080,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>16:17</t>
+          <t>16:18</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -19281,7 +19281,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>16:13</t>
+          <t>16:14</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -19482,7 +19482,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -19750,7 +19750,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -19951,12 +19951,12 @@
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="I292" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="J292" t="inlineStr">
@@ -20018,12 +20018,12 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="J293" t="inlineStr">
@@ -20090,7 +20090,7 @@
       </c>
       <c r="I294" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="J294" t="inlineStr">
@@ -20157,7 +20157,7 @@
       </c>
       <c r="I295" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="J295" t="inlineStr">
@@ -20219,12 +20219,12 @@
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="I296" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="J296" t="inlineStr">
@@ -20286,12 +20286,12 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="J297" t="inlineStr">
@@ -20358,7 +20358,7 @@
       </c>
       <c r="I298" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="J298" t="inlineStr">
@@ -20621,7 +20621,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:49</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -20688,7 +20688,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -21492,7 +21492,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -21559,7 +21559,7 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
@@ -21827,7 +21827,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
@@ -22229,7 +22229,7 @@
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="I326" t="inlineStr">
@@ -22363,7 +22363,7 @@
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="I328" t="inlineStr">
@@ -22497,7 +22497,7 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
@@ -22698,7 +22698,7 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="I333" t="inlineStr">
@@ -22899,7 +22899,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>14:23</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -24909,7 +24909,7 @@
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="I366" t="inlineStr">
@@ -25311,7 +25311,7 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:37</t>
         </is>
       </c>
       <c r="I372" t="inlineStr">
@@ -25378,7 +25378,7 @@
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>14:39</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="I373" t="inlineStr">
@@ -25914,7 +25914,7 @@
       </c>
       <c r="H381" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="I381" t="inlineStr">
@@ -25981,7 +25981,7 @@
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="I382" t="inlineStr">
@@ -26048,7 +26048,7 @@
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t>14:49</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="I383" t="inlineStr">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>14:49</t>
         </is>
       </c>
       <c r="I384" t="inlineStr">
@@ -26584,7 +26584,7 @@
       </c>
       <c r="H391" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="I391" t="inlineStr">
@@ -26651,7 +26651,7 @@
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
@@ -26718,7 +26718,7 @@
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="I393" t="inlineStr">
@@ -27120,7 +27120,7 @@
       </c>
       <c r="H399" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="I399" t="inlineStr">
@@ -27187,7 +27187,7 @@
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>15:08</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="I400" t="inlineStr">
@@ -27254,7 +27254,7 @@
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>15:09</t>
+          <t>15:08</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
@@ -27857,7 +27857,7 @@
       </c>
       <c r="H410" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="I410" t="inlineStr">
@@ -27924,7 +27924,7 @@
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="I411" t="inlineStr">
@@ -27991,7 +27991,7 @@
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>15:21</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="I412" t="inlineStr">
@@ -28058,7 +28058,7 @@
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
@@ -28125,7 +28125,7 @@
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
@@ -28192,7 +28192,7 @@
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="I415" t="inlineStr">
@@ -28259,7 +28259,7 @@
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="I416" t="inlineStr">
@@ -28326,7 +28326,7 @@
       </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="I417" t="inlineStr">
@@ -28393,7 +28393,7 @@
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="I418" t="inlineStr">
@@ -28460,7 +28460,7 @@
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
@@ -28527,7 +28527,7 @@
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>15:29</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
@@ -28594,7 +28594,7 @@
       </c>
       <c r="H421" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:29</t>
         </is>
       </c>
       <c r="I421" t="inlineStr">
@@ -29063,7 +29063,7 @@
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>15:36</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="I428" t="inlineStr">
@@ -29130,7 +29130,7 @@
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>15:37</t>
+          <t>15:36</t>
         </is>
       </c>
       <c r="I429" t="inlineStr">
@@ -29465,7 +29465,7 @@
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="I434" t="inlineStr">
@@ -29733,7 +29733,7 @@
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="I438" t="inlineStr">
@@ -30001,7 +30001,7 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
@@ -30202,7 +30202,7 @@
       </c>
       <c r="H445" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="I445" t="inlineStr">
@@ -30537,7 +30537,7 @@
       </c>
       <c r="H450" t="inlineStr">
         <is>
-          <t>16:52</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="I450" t="inlineStr">
@@ -30872,7 +30872,7 @@
       </c>
       <c r="H455" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:54</t>
         </is>
       </c>
       <c r="I455" t="inlineStr">
@@ -31006,7 +31006,7 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="I457" t="inlineStr">
@@ -31676,12 +31676,12 @@
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="I467" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="J467" t="inlineStr">
@@ -31748,7 +31748,7 @@
       </c>
       <c r="I468" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="J468" t="inlineStr">
@@ -31810,12 +31810,12 @@
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>17:02</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="I469" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="J469" t="inlineStr">
@@ -31882,7 +31882,7 @@
       </c>
       <c r="I470" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="J470" t="inlineStr">
@@ -31944,12 +31944,12 @@
       </c>
       <c r="H471" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>17:02</t>
         </is>
       </c>
       <c r="I471" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="J471" t="inlineStr">
@@ -32016,7 +32016,7 @@
       </c>
       <c r="I472" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="J472" t="inlineStr">
@@ -32083,7 +32083,7 @@
       </c>
       <c r="I473" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="J473" t="inlineStr">
@@ -32279,7 +32279,7 @@
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="I476" t="inlineStr">
@@ -32413,7 +32413,7 @@
       </c>
       <c r="H478" t="inlineStr">
         <is>
-          <t>17:06</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="I478" t="inlineStr">
@@ -32748,7 +32748,7 @@
       </c>
       <c r="H483" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="I483" t="inlineStr">
@@ -33284,7 +33284,7 @@
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="I491" t="inlineStr">
@@ -33820,7 +33820,7 @@
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:13</t>
         </is>
       </c>
       <c r="I499" t="inlineStr">
@@ -34021,7 +34021,7 @@
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="I502" t="inlineStr">
@@ -34959,7 +34959,7 @@
       </c>
       <c r="H516" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>17:19</t>
         </is>
       </c>
       <c r="I516" t="inlineStr">
@@ -35160,7 +35160,7 @@
       </c>
       <c r="H519" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="I519" t="inlineStr">
@@ -37036,7 +37036,7 @@
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>17:27</t>
+          <t>17:28</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
@@ -38510,7 +38510,7 @@
       </c>
       <c r="H569" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:27</t>
         </is>
       </c>
       <c r="I569" t="inlineStr">
@@ -39113,7 +39113,7 @@
       </c>
       <c r="H578" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="I578" t="inlineStr">
@@ -39515,7 +39515,7 @@
       </c>
       <c r="H584" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="I584" t="inlineStr">
@@ -39850,7 +39850,7 @@
       </c>
       <c r="H589" t="inlineStr">
         <is>
-          <t>17:17</t>
+          <t>17:18</t>
         </is>
       </c>
       <c r="I589" t="inlineStr">
@@ -40051,7 +40051,7 @@
       </c>
       <c r="H592" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="I592" t="inlineStr">
@@ -40319,7 +40319,7 @@
       </c>
       <c r="H596" t="inlineStr">
         <is>
-          <t>17:12</t>
+          <t>17:13</t>
         </is>
       </c>
       <c r="I596" t="inlineStr">
@@ -40788,7 +40788,7 @@
       </c>
       <c r="H603" t="inlineStr">
         <is>
-          <t>17:06</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="I603" t="inlineStr">
@@ -40855,7 +40855,7 @@
       </c>
       <c r="H604" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:06</t>
         </is>
       </c>
       <c r="I604" t="inlineStr">
@@ -40922,7 +40922,7 @@
       </c>
       <c r="H605" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="I605" t="inlineStr">
@@ -40989,7 +40989,7 @@
       </c>
       <c r="H606" t="inlineStr">
         <is>
-          <t>17:03</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="I606" t="inlineStr">
@@ -41056,7 +41056,7 @@
       </c>
       <c r="H607" t="inlineStr">
         <is>
-          <t>17:02</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="I607" t="inlineStr">
@@ -41123,7 +41123,7 @@
       </c>
       <c r="H608" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:02</t>
         </is>
       </c>
       <c r="I608" t="inlineStr">
@@ -41190,7 +41190,7 @@
       </c>
       <c r="H609" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="I609" t="inlineStr">
@@ -41257,7 +41257,7 @@
       </c>
       <c r="H610" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="I610" t="inlineStr">
@@ -41324,7 +41324,7 @@
       </c>
       <c r="H611" t="inlineStr">
         <is>
-          <t>16:58</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="I611" t="inlineStr">
@@ -41391,7 +41391,7 @@
       </c>
       <c r="H612" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="I612" t="inlineStr">
@@ -41860,7 +41860,7 @@
       </c>
       <c r="H619" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="I619" t="inlineStr">
@@ -41927,7 +41927,7 @@
       </c>
       <c r="H620" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:49</t>
         </is>
       </c>
       <c r="I620" t="inlineStr">
@@ -42195,7 +42195,7 @@
       </c>
       <c r="H624" t="inlineStr">
         <is>
-          <t>16:43</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="I624" t="inlineStr">
@@ -42463,7 +42463,7 @@
       </c>
       <c r="H628" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:39</t>
         </is>
       </c>
       <c r="I628" t="inlineStr">
@@ -42731,7 +42731,7 @@
       </c>
       <c r="H632" t="inlineStr">
         <is>
-          <t>16:33</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="I632" t="inlineStr">
@@ -43200,7 +43200,7 @@
       </c>
       <c r="H639" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="I639" t="inlineStr">
@@ -43401,7 +43401,7 @@
       </c>
       <c r="H642" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>16:21</t>
         </is>
       </c>
       <c r="I642" t="inlineStr">
@@ -43602,7 +43602,7 @@
       </c>
       <c r="H645" t="inlineStr">
         <is>
-          <t>16:16</t>
+          <t>16:17</t>
         </is>
       </c>
       <c r="I645" t="inlineStr">
@@ -43803,7 +43803,7 @@
       </c>
       <c r="H648" t="inlineStr">
         <is>
-          <t>16:12</t>
+          <t>16:13</t>
         </is>
       </c>
       <c r="I648" t="inlineStr">
@@ -44004,7 +44004,7 @@
       </c>
       <c r="H651" t="inlineStr">
         <is>
-          <t>16:08</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="I651" t="inlineStr">
@@ -44272,7 +44272,7 @@
       </c>
       <c r="H655" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="I655" t="inlineStr">
@@ -44473,7 +44473,7 @@
       </c>
       <c r="H658" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="I658" t="inlineStr">
@@ -44540,7 +44540,7 @@
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="I659" t="inlineStr">
@@ -44808,7 +44808,7 @@
       </c>
       <c r="H663" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="I663" t="inlineStr">
@@ -45210,7 +45210,7 @@
       </c>
       <c r="H669" t="inlineStr">
         <is>
-          <t>15:46</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="I669" t="inlineStr">
@@ -45277,12 +45277,12 @@
       </c>
       <c r="H670" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:46</t>
         </is>
       </c>
       <c r="I670" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="J670" t="inlineStr">
@@ -45344,12 +45344,12 @@
       </c>
       <c r="H671" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="I671" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="J671" t="inlineStr">
@@ -45411,12 +45411,12 @@
       </c>
       <c r="H672" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="I672" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="J672" t="inlineStr">
@@ -45483,7 +45483,7 @@
       </c>
       <c r="I673" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="J673" t="inlineStr">
@@ -45550,7 +45550,7 @@
       </c>
       <c r="I674" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="J674" t="inlineStr">
@@ -45617,7 +45617,7 @@
       </c>
       <c r="I675" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="J675" t="inlineStr">
@@ -45684,7 +45684,7 @@
       </c>
       <c r="I676" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="J676" t="inlineStr">
@@ -45746,7 +45746,7 @@
       </c>
       <c r="H677" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:39</t>
         </is>
       </c>
       <c r="I677" t="inlineStr">
@@ -45813,7 +45813,7 @@
       </c>
       <c r="H678" t="inlineStr">
         <is>
-          <t>14:37</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="I678" t="inlineStr">
@@ -45880,7 +45880,7 @@
       </c>
       <c r="H679" t="inlineStr">
         <is>
-          <t>14:36</t>
+          <t>14:37</t>
         </is>
       </c>
       <c r="I679" t="inlineStr">
@@ -45947,7 +45947,7 @@
       </c>
       <c r="H680" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="I680" t="inlineStr">
@@ -46282,7 +46282,7 @@
       </c>
       <c r="H685" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="I685" t="inlineStr">
@@ -46483,7 +46483,7 @@
       </c>
       <c r="H688" t="inlineStr">
         <is>
-          <t>14:29</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="I688" t="inlineStr">
@@ -46684,7 +46684,7 @@
       </c>
       <c r="H691" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="I691" t="inlineStr">
@@ -46818,7 +46818,7 @@
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="I693" t="inlineStr">
@@ -47153,7 +47153,7 @@
       </c>
       <c r="H698" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="I698" t="inlineStr">
@@ -47421,7 +47421,7 @@
       </c>
       <c r="H702" t="inlineStr">
         <is>
-          <t>14:23</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="I702" t="inlineStr">
@@ -49297,7 +49297,7 @@
       </c>
       <c r="H730" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="I730" t="inlineStr">
@@ -49632,7 +49632,7 @@
       </c>
       <c r="H735" t="inlineStr">
         <is>
-          <t>14:36</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="I735" t="inlineStr">
@@ -49699,7 +49699,7 @@
       </c>
       <c r="H736" t="inlineStr">
         <is>
-          <t>14:37</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="I736" t="inlineStr">
@@ -50637,7 +50637,7 @@
       </c>
       <c r="H750" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="I750" t="inlineStr">
@@ -50704,7 +50704,7 @@
       </c>
       <c r="H751" t="inlineStr">
         <is>
-          <t>14:52</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="I751" t="inlineStr">
@@ -50771,7 +50771,7 @@
       </c>
       <c r="H752" t="inlineStr">
         <is>
-          <t>14:53</t>
+          <t>14:52</t>
         </is>
       </c>
       <c r="I752" t="inlineStr">
@@ -51240,7 +51240,7 @@
       </c>
       <c r="H759" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="I759" t="inlineStr">
@@ -51307,7 +51307,7 @@
       </c>
       <c r="H760" t="inlineStr">
         <is>
-          <t>15:02</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="I760" t="inlineStr">
@@ -51776,7 +51776,7 @@
       </c>
       <c r="H767" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:09</t>
         </is>
       </c>
       <c r="I767" t="inlineStr">
@@ -51843,7 +51843,7 @@
       </c>
       <c r="H768" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="I768" t="inlineStr">
@@ -51910,7 +51910,7 @@
       </c>
       <c r="H769" t="inlineStr">
         <is>
-          <t>15:12</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="I769" t="inlineStr">
@@ -53451,7 +53451,7 @@
       </c>
       <c r="H792" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="I792" t="inlineStr">
@@ -53518,7 +53518,7 @@
       </c>
       <c r="H793" t="inlineStr">
         <is>
-          <t>15:36</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="I793" t="inlineStr">
@@ -53853,7 +53853,7 @@
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:39</t>
         </is>
       </c>
       <c r="I798" t="inlineStr">
@@ -54188,7 +54188,7 @@
       </c>
       <c r="H803" t="inlineStr">
         <is>
-          <t>15:44</t>
+          <t>15:43</t>
         </is>
       </c>
       <c r="I803" t="inlineStr">
@@ -54389,7 +54389,7 @@
       </c>
       <c r="H806" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="I806" t="inlineStr">
@@ -54590,7 +54590,7 @@
       </c>
       <c r="H809" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="I809" t="inlineStr">
@@ -54791,7 +54791,7 @@
       </c>
       <c r="H812" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>16:49</t>
         </is>
       </c>
       <c r="I812" t="inlineStr">
@@ -54992,7 +54992,7 @@
       </c>
       <c r="H815" t="inlineStr">
         <is>
-          <t>16:52</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="I815" t="inlineStr">
@@ -55461,7 +55461,7 @@
       </c>
       <c r="H822" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="I822" t="inlineStr">
@@ -55595,7 +55595,7 @@
       </c>
       <c r="H824" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="I824" t="inlineStr">
@@ -55729,7 +55729,7 @@
       </c>
       <c r="H826" t="inlineStr">
         <is>
-          <t>16:58</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="I826" t="inlineStr">
@@ -55863,7 +55863,7 @@
       </c>
       <c r="H828" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="I828" t="inlineStr">
@@ -55997,7 +55997,7 @@
       </c>
       <c r="H830" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="I830" t="inlineStr">
@@ -56131,7 +56131,7 @@
       </c>
       <c r="H832" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="I832" t="inlineStr">
@@ -56265,7 +56265,7 @@
       </c>
       <c r="H834" t="inlineStr">
         <is>
-          <t>17:02</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="I834" t="inlineStr">
@@ -56734,7 +56734,7 @@
       </c>
       <c r="H841" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="I841" t="inlineStr">
@@ -57069,7 +57069,7 @@
       </c>
       <c r="H846" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>17:06</t>
         </is>
       </c>
       <c r="I846" t="inlineStr">
@@ -57404,7 +57404,7 @@
       </c>
       <c r="H851" t="inlineStr">
         <is>
-          <t>17:09</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="I851" t="inlineStr">
@@ -57940,7 +57940,7 @@
       </c>
       <c r="H859" t="inlineStr">
         <is>
-          <t>17:12</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="I859" t="inlineStr">
@@ -58476,7 +58476,7 @@
       </c>
       <c r="H867" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="I867" t="inlineStr">
@@ -58677,7 +58677,7 @@
       </c>
       <c r="H870" t="inlineStr">
         <is>
-          <t>17:16</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="I870" t="inlineStr">
@@ -62630,7 +62630,7 @@
       </c>
       <c r="H929" t="inlineStr">
         <is>
-          <t>17:27</t>
+          <t>17:28</t>
         </is>
       </c>
       <c r="I929" t="inlineStr">
@@ -62965,7 +62965,7 @@
       </c>
       <c r="H934" t="inlineStr">
         <is>
-          <t>17:26</t>
+          <t>17:27</t>
         </is>
       </c>
       <c r="I934" t="inlineStr">
@@ -64104,7 +64104,7 @@
       </c>
       <c r="H951" t="inlineStr">
         <is>
-          <t>17:19</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="I951" t="inlineStr">
@@ -64707,7 +64707,7 @@
       </c>
       <c r="H960" t="inlineStr">
         <is>
-          <t>17:13</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="I960" t="inlineStr">
@@ -65109,7 +65109,7 @@
       </c>
       <c r="H966" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:09</t>
         </is>
       </c>
       <c r="I966" t="inlineStr">
@@ -65176,7 +65176,7 @@
       </c>
       <c r="H967" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="I967" t="inlineStr">
@@ -65913,7 +65913,7 @@
       </c>
       <c r="H978" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="I978" t="inlineStr">
@@ -65980,7 +65980,7 @@
       </c>
       <c r="H979" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="I979" t="inlineStr">
@@ -66047,7 +66047,7 @@
       </c>
       <c r="H980" t="inlineStr">
         <is>
-          <t>16:54</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="I980" t="inlineStr">
@@ -66449,7 +66449,7 @@
       </c>
       <c r="H986" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="I986" t="inlineStr">
@@ -66784,7 +66784,7 @@
       </c>
       <c r="H991" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:42</t>
         </is>
       </c>
       <c r="I991" t="inlineStr">
@@ -67052,7 +67052,7 @@
       </c>
       <c r="H995" t="inlineStr">
         <is>
-          <t>16:36</t>
+          <t>16:37</t>
         </is>
       </c>
       <c r="I995" t="inlineStr">
@@ -67253,7 +67253,7 @@
       </c>
       <c r="H998" t="inlineStr">
         <is>
-          <t>16:32</t>
+          <t>16:33</t>
         </is>
       </c>
       <c r="I998" t="inlineStr">
@@ -67722,7 +67722,7 @@
       </c>
       <c r="H1005" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="I1005" t="inlineStr">
@@ -67923,7 +67923,7 @@
       </c>
       <c r="H1008" t="inlineStr">
         <is>
-          <t>16:19</t>
+          <t>16:20</t>
         </is>
       </c>
       <c r="I1008" t="inlineStr">
@@ -68124,7 +68124,7 @@
       </c>
       <c r="H1011" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="I1011" t="inlineStr">
@@ -68325,7 +68325,7 @@
       </c>
       <c r="H1014" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:12</t>
         </is>
       </c>
       <c r="I1014" t="inlineStr">
@@ -68526,7 +68526,7 @@
       </c>
       <c r="H1017" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:08</t>
         </is>
       </c>
       <c r="I1017" t="inlineStr">
@@ -68794,7 +68794,7 @@
       </c>
       <c r="H1021" t="inlineStr">
         <is>
-          <t>16:02</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="I1021" t="inlineStr">
@@ -69062,7 +69062,7 @@
       </c>
       <c r="H1025" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="I1025" t="inlineStr">
@@ -69330,7 +69330,7 @@
       </c>
       <c r="H1029" t="inlineStr">
         <is>
-          <t>15:52</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="I1029" t="inlineStr">
@@ -69397,7 +69397,7 @@
       </c>
       <c r="H1030" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:52</t>
         </is>
       </c>
       <c r="I1030" t="inlineStr">
@@ -69866,7 +69866,7 @@
       </c>
       <c r="H1037" t="inlineStr">
         <is>
-          <t>15:43</t>
+          <t>15:44</t>
         </is>
       </c>
       <c r="I1037" t="inlineStr">
@@ -69933,7 +69933,7 @@
       </c>
       <c r="H1038" t="inlineStr">
         <is>
-          <t>15:42</t>
+          <t>15:43</t>
         </is>
       </c>
       <c r="I1038" t="inlineStr">
@@ -70000,7 +70000,7 @@
       </c>
       <c r="H1039" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="I1039" t="inlineStr">
@@ -70067,7 +70067,7 @@
       </c>
       <c r="H1040" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="I1040" t="inlineStr">
@@ -70134,7 +70134,7 @@
       </c>
       <c r="H1041" t="inlineStr">
         <is>
-          <t>15:39</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="I1041" t="inlineStr">
@@ -70201,7 +70201,7 @@
       </c>
       <c r="H1042" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:39</t>
         </is>
       </c>
       <c r="I1042" t="inlineStr">
@@ -70268,7 +70268,7 @@
       </c>
       <c r="H1043" t="inlineStr">
         <is>
-          <t>14:37</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="I1043" t="inlineStr">
@@ -70670,7 +70670,7 @@
       </c>
       <c r="H1049" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="I1049" t="inlineStr">
@@ -70938,7 +70938,7 @@
       </c>
       <c r="H1053" t="inlineStr">
         <is>
-          <t>14:29</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="I1053" t="inlineStr">
@@ -71072,7 +71072,7 @@
       </c>
       <c r="H1055" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:29</t>
         </is>
       </c>
       <c r="I1055" t="inlineStr">
@@ -71608,7 +71608,7 @@
       </c>
       <c r="H1063" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="I1063" t="inlineStr">
@@ -71876,7 +71876,7 @@
       </c>
       <c r="H1067" t="inlineStr">
         <is>
-          <t>14:23</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="I1067" t="inlineStr">
@@ -73350,7 +73350,7 @@
       </c>
       <c r="H1089" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="I1089" t="inlineStr">

</xml_diff>

<commit_message>
Seperate iqamah calc func added
</commit_message>
<xml_diff>
--- a/sync/prayer_db.xlsx
+++ b/sync/prayer_db.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>14:40</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1124,7 +1124,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:42</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>14:42</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>14:43</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1325,7 +1325,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:45</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1392,7 +1392,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>14:46</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2062,7 +2062,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:58</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>15:04</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:16</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3268,7 +3268,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>15:16</t>
+          <t>15:17</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>15:17</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -4072,7 +4072,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:29</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -4139,7 +4139,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>15:29</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4206,7 +4206,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:31</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>15:31</t>
+          <t>15:32</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>15:37</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5077,7 +5077,7 @@
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:42</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -5345,7 +5345,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>16:44</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5747,7 +5747,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:49</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -5948,7 +5948,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="H88" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:54</t>
         </is>
       </c>
       <c r="I88" t="inlineStr">
@@ -6417,7 +6417,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>16:54</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -7489,7 +7489,7 @@
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>17:02</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
@@ -7958,7 +7958,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:06</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -8628,7 +8628,7 @@
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>17:09</t>
+          <t>17:10</t>
         </is>
       </c>
       <c r="I123" t="inlineStr">
@@ -9365,7 +9365,7 @@
       </c>
       <c r="H134" t="inlineStr">
         <is>
-          <t>17:13</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -10102,7 +10102,7 @@
       </c>
       <c r="H145" t="inlineStr">
         <is>
-          <t>17:17</t>
+          <t>17:18</t>
         </is>
       </c>
       <c r="I145" t="inlineStr">
@@ -10303,7 +10303,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>17:18</t>
+          <t>17:19</t>
         </is>
       </c>
       <c r="I148" t="inlineStr">
@@ -10906,7 +10906,7 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="I157" t="inlineStr">
@@ -14792,7 +14792,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
@@ -14926,7 +14926,7 @@
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
@@ -15931,7 +15931,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>17:12</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="I232" t="inlineStr">
@@ -17338,7 +17338,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="I253" t="inlineStr">
@@ -17673,7 +17673,7 @@
       </c>
       <c r="H258" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="I258" t="inlineStr">
@@ -17941,7 +17941,7 @@
       </c>
       <c r="H262" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:39</t>
         </is>
       </c>
       <c r="I262" t="inlineStr">
@@ -18209,7 +18209,7 @@
       </c>
       <c r="H266" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:34</t>
         </is>
       </c>
       <c r="I266" t="inlineStr">
@@ -18678,7 +18678,7 @@
       </c>
       <c r="H273" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="I273" t="inlineStr">
@@ -18879,7 +18879,7 @@
       </c>
       <c r="H276" t="inlineStr">
         <is>
-          <t>16:22</t>
+          <t>16:21</t>
         </is>
       </c>
       <c r="I276" t="inlineStr">
@@ -19080,7 +19080,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>16:18</t>
+          <t>16:17</t>
         </is>
       </c>
       <c r="I279" t="inlineStr">
@@ -19281,7 +19281,7 @@
       </c>
       <c r="H282" t="inlineStr">
         <is>
-          <t>16:14</t>
+          <t>16:13</t>
         </is>
       </c>
       <c r="I282" t="inlineStr">
@@ -19482,7 +19482,7 @@
       </c>
       <c r="H285" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="I285" t="inlineStr">
@@ -19750,7 +19750,7 @@
       </c>
       <c r="H289" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>16:04</t>
         </is>
       </c>
       <c r="I289" t="inlineStr">
@@ -20018,7 +20018,7 @@
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="I293" t="inlineStr">
@@ -20286,7 +20286,7 @@
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>15:55</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="I297" t="inlineStr">
@@ -20621,7 +20621,7 @@
       </c>
       <c r="H302" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="I302" t="inlineStr">
@@ -20688,7 +20688,7 @@
       </c>
       <c r="H303" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="I303" t="inlineStr">
@@ -21492,7 +21492,7 @@
       </c>
       <c r="H315" t="inlineStr">
         <is>
-          <t>14:36</t>
+          <t>14:35</t>
         </is>
       </c>
       <c r="I315" t="inlineStr">
@@ -21559,7 +21559,7 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:34</t>
         </is>
       </c>
       <c r="I316" t="inlineStr">
@@ -21827,7 +21827,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
@@ -22229,7 +22229,7 @@
       </c>
       <c r="H326" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="I326" t="inlineStr">
@@ -22363,7 +22363,7 @@
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="I328" t="inlineStr">
@@ -22497,7 +22497,7 @@
       </c>
       <c r="H330" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="I330" t="inlineStr">
@@ -22698,7 +22698,7 @@
       </c>
       <c r="H333" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="I333" t="inlineStr">
@@ -22899,7 +22899,7 @@
       </c>
       <c r="H336" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="I336" t="inlineStr">
@@ -24909,7 +24909,7 @@
       </c>
       <c r="H366" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="I366" t="inlineStr">
@@ -25311,7 +25311,7 @@
       </c>
       <c r="H372" t="inlineStr">
         <is>
-          <t>14:37</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="I372" t="inlineStr">
@@ -25378,7 +25378,7 @@
       </c>
       <c r="H373" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:39</t>
         </is>
       </c>
       <c r="I373" t="inlineStr">
@@ -25981,7 +25981,7 @@
       </c>
       <c r="H382" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="I382" t="inlineStr">
@@ -26048,7 +26048,7 @@
       </c>
       <c r="H383" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:49</t>
         </is>
       </c>
       <c r="I383" t="inlineStr">
@@ -26115,7 +26115,7 @@
       </c>
       <c r="H384" t="inlineStr">
         <is>
-          <t>14:49</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="I384" t="inlineStr">
@@ -26651,7 +26651,7 @@
       </c>
       <c r="H392" t="inlineStr">
         <is>
-          <t>14:58</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="I392" t="inlineStr">
@@ -26718,7 +26718,7 @@
       </c>
       <c r="H393" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="I393" t="inlineStr">
@@ -27187,7 +27187,7 @@
       </c>
       <c r="H400" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:08</t>
         </is>
       </c>
       <c r="I400" t="inlineStr">
@@ -27254,7 +27254,7 @@
       </c>
       <c r="H401" t="inlineStr">
         <is>
-          <t>15:08</t>
+          <t>15:09</t>
         </is>
       </c>
       <c r="I401" t="inlineStr">
@@ -27924,7 +27924,7 @@
       </c>
       <c r="H411" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="I411" t="inlineStr">
@@ -27991,7 +27991,7 @@
       </c>
       <c r="H412" t="inlineStr">
         <is>
-          <t>15:20</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="I412" t="inlineStr">
@@ -28058,7 +28058,7 @@
       </c>
       <c r="H413" t="inlineStr">
         <is>
-          <t>15:21</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="I413" t="inlineStr">
@@ -28125,7 +28125,7 @@
       </c>
       <c r="H414" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="I414" t="inlineStr">
@@ -28192,7 +28192,7 @@
       </c>
       <c r="H415" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="I415" t="inlineStr">
@@ -28259,7 +28259,7 @@
       </c>
       <c r="H416" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="I416" t="inlineStr">
@@ -28326,7 +28326,7 @@
       </c>
       <c r="H417" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="I417" t="inlineStr">
@@ -28393,7 +28393,7 @@
       </c>
       <c r="H418" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="I418" t="inlineStr">
@@ -28460,7 +28460,7 @@
       </c>
       <c r="H419" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="I419" t="inlineStr">
@@ -28527,7 +28527,7 @@
       </c>
       <c r="H420" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:29</t>
         </is>
       </c>
       <c r="I420" t="inlineStr">
@@ -29063,7 +29063,7 @@
       </c>
       <c r="H428" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:36</t>
         </is>
       </c>
       <c r="I428" t="inlineStr">
@@ -29130,7 +29130,7 @@
       </c>
       <c r="H429" t="inlineStr">
         <is>
-          <t>15:36</t>
+          <t>15:37</t>
         </is>
       </c>
       <c r="I429" t="inlineStr">
@@ -29465,7 +29465,7 @@
       </c>
       <c r="H434" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="I434" t="inlineStr">
@@ -29733,7 +29733,7 @@
       </c>
       <c r="H438" t="inlineStr">
         <is>
-          <t>16:43</t>
+          <t>16:44</t>
         </is>
       </c>
       <c r="I438" t="inlineStr">
@@ -30001,7 +30001,7 @@
       </c>
       <c r="H442" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="I442" t="inlineStr">
@@ -30202,7 +30202,7 @@
       </c>
       <c r="H445" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:49</t>
         </is>
       </c>
       <c r="I445" t="inlineStr">
@@ -30537,7 +30537,7 @@
       </c>
       <c r="H450" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="I450" t="inlineStr">
@@ -30872,7 +30872,7 @@
       </c>
       <c r="H455" t="inlineStr">
         <is>
-          <t>16:54</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="I455" t="inlineStr">
@@ -31006,7 +31006,7 @@
       </c>
       <c r="H457" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="I457" t="inlineStr">
@@ -31676,12 +31676,12 @@
       </c>
       <c r="H467" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="I467" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="J467" t="inlineStr">
@@ -31748,7 +31748,7 @@
       </c>
       <c r="I468" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="J468" t="inlineStr">
@@ -31810,12 +31810,12 @@
       </c>
       <c r="H469" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:02</t>
         </is>
       </c>
       <c r="I469" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="J469" t="inlineStr">
@@ -31882,7 +31882,7 @@
       </c>
       <c r="I470" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="J470" t="inlineStr">
@@ -31949,7 +31949,7 @@
       </c>
       <c r="I471" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="J471" t="inlineStr">
@@ -32016,7 +32016,7 @@
       </c>
       <c r="I472" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="J472" t="inlineStr">
@@ -32083,7 +32083,7 @@
       </c>
       <c r="I473" t="inlineStr">
         <is>
-          <t>17:30</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="J473" t="inlineStr">
@@ -32279,7 +32279,7 @@
       </c>
       <c r="H476" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="I476" t="inlineStr">
@@ -33284,7 +33284,7 @@
       </c>
       <c r="H491" t="inlineStr">
         <is>
-          <t>17:10</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="I491" t="inlineStr">
@@ -33820,7 +33820,7 @@
       </c>
       <c r="H499" t="inlineStr">
         <is>
-          <t>17:13</t>
+          <t>17:14</t>
         </is>
       </c>
       <c r="I499" t="inlineStr">
@@ -34021,7 +34021,7 @@
       </c>
       <c r="H502" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="I502" t="inlineStr">
@@ -37036,7 +37036,7 @@
       </c>
       <c r="H547" t="inlineStr">
         <is>
-          <t>17:28</t>
+          <t>17:27</t>
         </is>
       </c>
       <c r="I547" t="inlineStr">
@@ -38510,7 +38510,7 @@
       </c>
       <c r="H569" t="inlineStr">
         <is>
-          <t>17:27</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="I569" t="inlineStr">
@@ -39113,7 +39113,7 @@
       </c>
       <c r="H578" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="I578" t="inlineStr">
@@ -39515,7 +39515,7 @@
       </c>
       <c r="H584" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:20</t>
         </is>
       </c>
       <c r="I584" t="inlineStr">
@@ -39850,7 +39850,7 @@
       </c>
       <c r="H589" t="inlineStr">
         <is>
-          <t>17:18</t>
+          <t>17:17</t>
         </is>
       </c>
       <c r="I589" t="inlineStr">
@@ -40051,7 +40051,7 @@
       </c>
       <c r="H592" t="inlineStr">
         <is>
-          <t>17:16</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="I592" t="inlineStr">
@@ -40319,7 +40319,7 @@
       </c>
       <c r="H596" t="inlineStr">
         <is>
-          <t>17:13</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="I596" t="inlineStr">
@@ -40788,7 +40788,7 @@
       </c>
       <c r="H603" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>17:06</t>
         </is>
       </c>
       <c r="I603" t="inlineStr">
@@ -40855,7 +40855,7 @@
       </c>
       <c r="H604" t="inlineStr">
         <is>
-          <t>17:06</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="I604" t="inlineStr">
@@ -40922,7 +40922,7 @@
       </c>
       <c r="H605" t="inlineStr">
         <is>
-          <t>17:05</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="I605" t="inlineStr">
@@ -40989,7 +40989,7 @@
       </c>
       <c r="H606" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="I606" t="inlineStr">
@@ -41190,7 +41190,7 @@
       </c>
       <c r="H609" t="inlineStr">
         <is>
-          <t>17:01</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="I609" t="inlineStr">
@@ -41257,7 +41257,7 @@
       </c>
       <c r="H610" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="I610" t="inlineStr">
@@ -41324,7 +41324,7 @@
       </c>
       <c r="H611" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="I611" t="inlineStr">
@@ -41391,7 +41391,7 @@
       </c>
       <c r="H612" t="inlineStr">
         <is>
-          <t>16:58</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="I612" t="inlineStr">
@@ -41860,7 +41860,7 @@
       </c>
       <c r="H619" t="inlineStr">
         <is>
-          <t>16:50</t>
+          <t>16:49</t>
         </is>
       </c>
       <c r="I619" t="inlineStr">
@@ -41927,7 +41927,7 @@
       </c>
       <c r="H620" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="I620" t="inlineStr">
@@ -42731,7 +42731,7 @@
       </c>
       <c r="H632" t="inlineStr">
         <is>
-          <t>16:34</t>
+          <t>16:33</t>
         </is>
       </c>
       <c r="I632" t="inlineStr">
@@ -43200,7 +43200,7 @@
       </c>
       <c r="H639" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="I639" t="inlineStr">
@@ -43401,7 +43401,7 @@
       </c>
       <c r="H642" t="inlineStr">
         <is>
-          <t>16:21</t>
+          <t>16:20</t>
         </is>
       </c>
       <c r="I642" t="inlineStr">
@@ -43602,7 +43602,7 @@
       </c>
       <c r="H645" t="inlineStr">
         <is>
-          <t>16:17</t>
+          <t>16:16</t>
         </is>
       </c>
       <c r="I645" t="inlineStr">
@@ -43803,7 +43803,7 @@
       </c>
       <c r="H648" t="inlineStr">
         <is>
-          <t>16:13</t>
+          <t>16:12</t>
         </is>
       </c>
       <c r="I648" t="inlineStr">
@@ -44272,7 +44272,7 @@
       </c>
       <c r="H655" t="inlineStr">
         <is>
-          <t>16:04</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="I655" t="inlineStr">
@@ -44540,7 +44540,7 @@
       </c>
       <c r="H659" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="I659" t="inlineStr">
@@ -44808,7 +44808,7 @@
       </c>
       <c r="H663" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:53</t>
         </is>
       </c>
       <c r="I663" t="inlineStr">
@@ -45277,12 +45277,12 @@
       </c>
       <c r="H670" t="inlineStr">
         <is>
-          <t>15:46</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="I670" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="J670" t="inlineStr">
@@ -45344,12 +45344,12 @@
       </c>
       <c r="H671" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>14:44</t>
         </is>
       </c>
       <c r="I671" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="J671" t="inlineStr">
@@ -45411,12 +45411,12 @@
       </c>
       <c r="H672" t="inlineStr">
         <is>
-          <t>14:44</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="I672" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="J672" t="inlineStr">
@@ -45483,7 +45483,7 @@
       </c>
       <c r="I673" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="J673" t="inlineStr">
@@ -45550,7 +45550,7 @@
       </c>
       <c r="I674" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="J674" t="inlineStr">
@@ -45617,7 +45617,7 @@
       </c>
       <c r="I675" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="J675" t="inlineStr">
@@ -45684,7 +45684,7 @@
       </c>
       <c r="I676" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="J676" t="inlineStr">
@@ -45746,7 +45746,7 @@
       </c>
       <c r="H677" t="inlineStr">
         <is>
-          <t>14:39</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="I677" t="inlineStr">
@@ -45813,7 +45813,7 @@
       </c>
       <c r="H678" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:37</t>
         </is>
       </c>
       <c r="I678" t="inlineStr">
@@ -45880,7 +45880,7 @@
       </c>
       <c r="H679" t="inlineStr">
         <is>
-          <t>14:37</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="I679" t="inlineStr">
@@ -46282,7 +46282,7 @@
       </c>
       <c r="H685" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:31</t>
         </is>
       </c>
       <c r="I685" t="inlineStr">
@@ -46483,7 +46483,7 @@
       </c>
       <c r="H688" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:29</t>
         </is>
       </c>
       <c r="I688" t="inlineStr">
@@ -46818,7 +46818,7 @@
       </c>
       <c r="H693" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="I693" t="inlineStr">
@@ -47153,7 +47153,7 @@
       </c>
       <c r="H698" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="I698" t="inlineStr">
@@ -47421,7 +47421,7 @@
       </c>
       <c r="H702" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="I702" t="inlineStr">
@@ -49297,7 +49297,7 @@
       </c>
       <c r="H730" t="inlineStr">
         <is>
-          <t>14:31</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="I730" t="inlineStr">
@@ -49632,7 +49632,7 @@
       </c>
       <c r="H735" t="inlineStr">
         <is>
-          <t>14:35</t>
+          <t>14:36</t>
         </is>
       </c>
       <c r="I735" t="inlineStr">
@@ -50637,7 +50637,7 @@
       </c>
       <c r="H750" t="inlineStr">
         <is>
-          <t>14:50</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="I750" t="inlineStr">
@@ -50704,7 +50704,7 @@
       </c>
       <c r="H751" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:52</t>
         </is>
       </c>
       <c r="I751" t="inlineStr">
@@ -50771,7 +50771,7 @@
       </c>
       <c r="H752" t="inlineStr">
         <is>
-          <t>14:52</t>
+          <t>14:53</t>
         </is>
       </c>
       <c r="I752" t="inlineStr">
@@ -51240,7 +51240,7 @@
       </c>
       <c r="H759" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="I759" t="inlineStr">
@@ -51307,7 +51307,7 @@
       </c>
       <c r="H760" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>15:02</t>
         </is>
       </c>
       <c r="I760" t="inlineStr">
@@ -51776,7 +51776,7 @@
       </c>
       <c r="H767" t="inlineStr">
         <is>
-          <t>15:09</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="I767" t="inlineStr">
@@ -51843,7 +51843,7 @@
       </c>
       <c r="H768" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="I768" t="inlineStr">
@@ -51910,7 +51910,7 @@
       </c>
       <c r="H769" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:12</t>
         </is>
       </c>
       <c r="I769" t="inlineStr">
@@ -53451,7 +53451,7 @@
       </c>
       <c r="H792" t="inlineStr">
         <is>
-          <t>15:34</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="I792" t="inlineStr">
@@ -53518,7 +53518,7 @@
       </c>
       <c r="H793" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:36</t>
         </is>
       </c>
       <c r="I793" t="inlineStr">
@@ -53853,7 +53853,7 @@
       </c>
       <c r="H798" t="inlineStr">
         <is>
-          <t>15:39</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="I798" t="inlineStr">
@@ -54389,7 +54389,7 @@
       </c>
       <c r="H806" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="I806" t="inlineStr">
@@ -54590,7 +54590,7 @@
       </c>
       <c r="H809" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="I809" t="inlineStr">
@@ -54791,7 +54791,7 @@
       </c>
       <c r="H812" t="inlineStr">
         <is>
-          <t>16:49</t>
+          <t>16:50</t>
         </is>
       </c>
       <c r="I812" t="inlineStr">
@@ -54992,7 +54992,7 @@
       </c>
       <c r="H815" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="I815" t="inlineStr">
@@ -55461,7 +55461,7 @@
       </c>
       <c r="H822" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="I822" t="inlineStr">
@@ -55595,7 +55595,7 @@
       </c>
       <c r="H824" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:57</t>
         </is>
       </c>
       <c r="I824" t="inlineStr">
@@ -55729,7 +55729,7 @@
       </c>
       <c r="H826" t="inlineStr">
         <is>
-          <t>16:57</t>
+          <t>16:58</t>
         </is>
       </c>
       <c r="I826" t="inlineStr">
@@ -55863,7 +55863,7 @@
       </c>
       <c r="H828" t="inlineStr">
         <is>
-          <t>16:58</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="I828" t="inlineStr">
@@ -55997,7 +55997,7 @@
       </c>
       <c r="H830" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="I830" t="inlineStr">
@@ -56131,7 +56131,7 @@
       </c>
       <c r="H832" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>17:01</t>
         </is>
       </c>
       <c r="I832" t="inlineStr">
@@ -56734,7 +56734,7 @@
       </c>
       <c r="H841" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:05</t>
         </is>
       </c>
       <c r="I841" t="inlineStr">
@@ -57069,7 +57069,7 @@
       </c>
       <c r="H846" t="inlineStr">
         <is>
-          <t>17:06</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="I846" t="inlineStr">
@@ -57404,7 +57404,7 @@
       </c>
       <c r="H851" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:09</t>
         </is>
       </c>
       <c r="I851" t="inlineStr">
@@ -57940,7 +57940,7 @@
       </c>
       <c r="H859" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="I859" t="inlineStr">
@@ -58476,7 +58476,7 @@
       </c>
       <c r="H867" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:15</t>
         </is>
       </c>
       <c r="I867" t="inlineStr">
@@ -58677,7 +58677,7 @@
       </c>
       <c r="H870" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>17:16</t>
         </is>
       </c>
       <c r="I870" t="inlineStr">
@@ -62630,7 +62630,7 @@
       </c>
       <c r="H929" t="inlineStr">
         <is>
-          <t>17:28</t>
+          <t>17:27</t>
         </is>
       </c>
       <c r="I929" t="inlineStr">
@@ -62965,7 +62965,7 @@
       </c>
       <c r="H934" t="inlineStr">
         <is>
-          <t>17:27</t>
+          <t>17:26</t>
         </is>
       </c>
       <c r="I934" t="inlineStr">
@@ -64104,7 +64104,7 @@
       </c>
       <c r="H951" t="inlineStr">
         <is>
-          <t>17:20</t>
+          <t>17:19</t>
         </is>
       </c>
       <c r="I951" t="inlineStr">
@@ -64707,7 +64707,7 @@
       </c>
       <c r="H960" t="inlineStr">
         <is>
-          <t>17:14</t>
+          <t>17:13</t>
         </is>
       </c>
       <c r="I960" t="inlineStr">
@@ -65109,7 +65109,7 @@
       </c>
       <c r="H966" t="inlineStr">
         <is>
-          <t>17:09</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="I966" t="inlineStr">
@@ -65176,7 +65176,7 @@
       </c>
       <c r="H967" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="I967" t="inlineStr">
@@ -65980,7 +65980,7 @@
       </c>
       <c r="H979" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="I979" t="inlineStr">
@@ -66047,7 +66047,7 @@
       </c>
       <c r="H980" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:54</t>
         </is>
       </c>
       <c r="I980" t="inlineStr">
@@ -66449,7 +66449,7 @@
       </c>
       <c r="H986" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="I986" t="inlineStr">
@@ -66784,7 +66784,7 @@
       </c>
       <c r="H991" t="inlineStr">
         <is>
-          <t>16:42</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="I991" t="inlineStr">
@@ -67052,7 +67052,7 @@
       </c>
       <c r="H995" t="inlineStr">
         <is>
-          <t>16:37</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="I995" t="inlineStr">
@@ -67253,7 +67253,7 @@
       </c>
       <c r="H998" t="inlineStr">
         <is>
-          <t>16:33</t>
+          <t>16:32</t>
         </is>
       </c>
       <c r="I998" t="inlineStr">
@@ -67722,7 +67722,7 @@
       </c>
       <c r="H1005" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="I1005" t="inlineStr">
@@ -67923,7 +67923,7 @@
       </c>
       <c r="H1008" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>16:19</t>
         </is>
       </c>
       <c r="I1008" t="inlineStr">
@@ -68124,7 +68124,7 @@
       </c>
       <c r="H1011" t="inlineStr">
         <is>
-          <t>16:16</t>
+          <t>16:15</t>
         </is>
       </c>
       <c r="I1011" t="inlineStr">
@@ -68325,7 +68325,7 @@
       </c>
       <c r="H1014" t="inlineStr">
         <is>
-          <t>16:12</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="I1014" t="inlineStr">
@@ -68794,7 +68794,7 @@
       </c>
       <c r="H1021" t="inlineStr">
         <is>
-          <t>16:03</t>
+          <t>16:02</t>
         </is>
       </c>
       <c r="I1021" t="inlineStr">
@@ -69062,7 +69062,7 @@
       </c>
       <c r="H1025" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="I1025" t="inlineStr">
@@ -69397,7 +69397,7 @@
       </c>
       <c r="H1030" t="inlineStr">
         <is>
-          <t>15:52</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="I1030" t="inlineStr">
@@ -69933,7 +69933,7 @@
       </c>
       <c r="H1038" t="inlineStr">
         <is>
-          <t>15:43</t>
+          <t>15:42</t>
         </is>
       </c>
       <c r="I1038" t="inlineStr">
@@ -70000,7 +70000,7 @@
       </c>
       <c r="H1039" t="inlineStr">
         <is>
-          <t>15:42</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="I1039" t="inlineStr">
@@ -70067,7 +70067,7 @@
       </c>
       <c r="H1040" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="I1040" t="inlineStr">
@@ -70134,7 +70134,7 @@
       </c>
       <c r="H1041" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:39</t>
         </is>
       </c>
       <c r="I1041" t="inlineStr">
@@ -70201,7 +70201,7 @@
       </c>
       <c r="H1042" t="inlineStr">
         <is>
-          <t>14:39</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="I1042" t="inlineStr">
@@ -70670,7 +70670,7 @@
       </c>
       <c r="H1049" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="I1049" t="inlineStr">
@@ -71072,7 +71072,7 @@
       </c>
       <c r="H1055" t="inlineStr">
         <is>
-          <t>14:29</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="I1055" t="inlineStr">
@@ -71608,7 +71608,7 @@
       </c>
       <c r="H1063" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:24</t>
         </is>
       </c>
       <c r="I1063" t="inlineStr">
@@ -71876,7 +71876,7 @@
       </c>
       <c r="H1067" t="inlineStr">
         <is>
-          <t>14:24</t>
+          <t>14:23</t>
         </is>
       </c>
       <c r="I1067" t="inlineStr">
@@ -73350,7 +73350,7 @@
       </c>
       <c r="H1089" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="I1089" t="inlineStr">

</xml_diff>